<commit_message>
G4D Book — R1.8.1
• Added explanation of collapse boundary instability near G4D ≈ −0.30
• Added physical interpretation for high positive G4D regime (supergiants)
• Improved conceptual diagram of G4D visibility regimes
• Added astrophysical anchors (Sun, Betelgeuse, 300 M☉ star)
• Improved figure layout and caption clarity
• Updated index
• Minor formatting corrections

Data / Model Updates
• Updated Excel datasets with revised Appendix B (AB) text descriptions

Fixes
• Minor formatting corrections
</commit_message>
<xml_diff>
--- a/data/G4D_master_equation_dataset.xlsx
+++ b/data/G4D_master_equation_dataset.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="2970" yWindow="140" windowWidth="25860" windowHeight="9090"/>
+    <workbookView xWindow="2970" yWindow="140" windowWidth="26990" windowHeight="18040"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -505,7 +505,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="116">
+  <cellXfs count="118">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -832,6 +832,12 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1698,7 +1704,7 @@
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>30</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>304800</xdr:colOff>
       <xdr:row>20</xdr:row>
       <xdr:rowOff>107949</xdr:rowOff>
@@ -1782,7 +1788,7 @@
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>30</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>304800</xdr:colOff>
       <xdr:row>20</xdr:row>
       <xdr:rowOff>107949</xdr:rowOff>
@@ -1866,7 +1872,7 @@
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>30</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>304800</xdr:colOff>
       <xdr:row>20</xdr:row>
       <xdr:rowOff>107949</xdr:rowOff>
@@ -1950,7 +1956,7 @@
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>30</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>304800</xdr:colOff>
       <xdr:row>25</xdr:row>
       <xdr:rowOff>109070</xdr:rowOff>
@@ -1992,7 +1998,7 @@
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>30</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>304800</xdr:colOff>
       <xdr:row>25</xdr:row>
       <xdr:rowOff>109070</xdr:rowOff>
@@ -2076,7 +2082,7 @@
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>30</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>304800</xdr:colOff>
       <xdr:row>25</xdr:row>
       <xdr:rowOff>109070</xdr:rowOff>
@@ -2160,7 +2166,7 @@
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>30</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>304800</xdr:colOff>
       <xdr:row>25</xdr:row>
       <xdr:rowOff>109070</xdr:rowOff>
@@ -2244,7 +2250,7 @@
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>30</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>304800</xdr:colOff>
       <xdr:row>25</xdr:row>
       <xdr:rowOff>109070</xdr:rowOff>
@@ -2328,7 +2334,7 @@
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>30</xdr:col>
+      <xdr:col>31</xdr:col>
       <xdr:colOff>304800</xdr:colOff>
       <xdr:row>25</xdr:row>
       <xdr:rowOff>109070</xdr:rowOff>
@@ -3744,16 +3750,17 @@
     <col min="18" max="18" width="16.7265625" hidden="1" customWidth="1"/>
     <col min="19" max="19" width="20.26953125" hidden="1" customWidth="1"/>
     <col min="20" max="20" width="11.81640625" hidden="1" customWidth="1"/>
-    <col min="21" max="21" width="0" hidden="1" customWidth="1"/>
+    <col min="21" max="21" width="8.7265625" customWidth="1"/>
     <col min="22" max="22" width="12.54296875" hidden="1" customWidth="1"/>
     <col min="23" max="23" width="16.1796875" hidden="1" customWidth="1"/>
     <col min="24" max="24" width="12.453125" hidden="1" customWidth="1"/>
     <col min="25" max="25" width="14.7265625" hidden="1" customWidth="1"/>
     <col min="26" max="26" width="18" hidden="1" customWidth="1"/>
     <col min="27" max="27" width="20.1796875" hidden="1" customWidth="1"/>
-    <col min="28" max="28" width="18" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="21.453125" bestFit="1" customWidth="1"/>
     <col min="29" max="29" width="8.36328125" hidden="1" customWidth="1"/>
-    <col min="30" max="30" width="12.7265625" hidden="1" customWidth="1"/>
+    <col min="30" max="30" width="9.7265625" hidden="1" customWidth="1"/>
+    <col min="31" max="31" width="0" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:30" ht="15" thickBot="1" x14ac:dyDescent="0.4">
@@ -3838,7 +3845,7 @@
       <c r="AA1" s="56" t="s">
         <v>25</v>
       </c>
-      <c r="AB1" s="56" t="s">
+      <c r="AB1" s="57" t="s">
         <v>23</v>
       </c>
       <c r="AC1" s="59" t="s">
@@ -3958,13 +3965,17 @@
 "Invisible (Black hole)"))))</f>
         <v>Invisible (Black hole)</v>
       </c>
-      <c r="AB2" s="104" t="str">
-        <f>IF(P2&gt;0,"Fully visible",
+      <c r="AB2" s="116" t="str">
+        <f>IF(U2&gt;=1,
+   IF(E2&gt;=100000,"Supermassive Black hole",
+   IF(E2&gt;=100,"Intermediate Black hole",
+   "Stellar Black hole")),
+IF(P2&gt;0,"Fully visible",
 IF(P2&gt;-0.26,"Partial visible",
 IF(ABS(P2+0.3)&lt;=0.02,"Collapse boundary",
 IF(P2&gt;-0.32,"Collapse transition",
-"Invisible (Black hole)"))))</f>
-        <v>Invisible (Black hole)</v>
+"Invisible (geometric)")))))</f>
+        <v>Supermassive Black hole</v>
       </c>
       <c r="AC2" s="106">
         <f>E2*1.788E+47</f>
@@ -4083,13 +4094,17 @@
 "Invisible (Black hole)"))))</f>
         <v>Invisible (Black hole)</v>
       </c>
-      <c r="AB3" s="104" t="str">
-        <f t="shared" ref="AB3:AB39" si="11">IF(P3&gt;0,"Fully visible",
+      <c r="AB3" s="116" t="str">
+        <f t="shared" ref="AB3:AB39" si="11">IF(U3&gt;=1,
+   IF(E3&gt;=100000,"Supermassive Black hole",
+   IF(E3&gt;=100,"Intermediate Black hole",
+   "Stellar Black hole")),
+IF(P3&gt;0,"Fully visible",
 IF(P3&gt;-0.26,"Partial visible",
 IF(ABS(P3+0.3)&lt;=0.02,"Collapse boundary",
 IF(P3&gt;-0.32,"Collapse transition",
-"Invisible (Black hole)"))))</f>
-        <v>Invisible (Black hole)</v>
+"Invisible (geometric)")))))</f>
+        <v>Supermassive Black hole</v>
       </c>
       <c r="AC3" s="110">
         <f t="shared" ref="AC3:AC39" si="12">E3*1.788E+47</f>
@@ -4201,9 +4216,9 @@
         <f t="shared" si="10"/>
         <v>Invisible (Black hole)</v>
       </c>
-      <c r="AB4" s="104" t="str">
+      <c r="AB4" s="116" t="str">
         <f t="shared" si="11"/>
-        <v>Invisible (Black hole)</v>
+        <v>Stellar Black hole</v>
       </c>
       <c r="AC4" s="110">
         <f t="shared" si="12"/>
@@ -4315,9 +4330,9 @@
         <f t="shared" si="10"/>
         <v>Invisible (Black hole)</v>
       </c>
-      <c r="AB5" s="104" t="str">
+      <c r="AB5" s="116" t="str">
         <f t="shared" si="11"/>
-        <v>Invisible (Black hole)</v>
+        <v>Stellar Black hole</v>
       </c>
       <c r="AC5" s="110">
         <f t="shared" si="12"/>
@@ -4429,9 +4444,9 @@
         <f t="shared" si="10"/>
         <v>Invisible (Black hole)</v>
       </c>
-      <c r="AB6" s="104" t="str">
+      <c r="AB6" s="116" t="str">
         <f t="shared" si="11"/>
-        <v>Invisible (Black hole)</v>
+        <v>Invisible (geometric)</v>
       </c>
       <c r="AC6" s="110">
         <f t="shared" si="12"/>
@@ -4543,9 +4558,9 @@
         <f t="shared" si="10"/>
         <v>Invisible (Black hole)</v>
       </c>
-      <c r="AB7" s="104" t="str">
+      <c r="AB7" s="116" t="str">
         <f t="shared" si="11"/>
-        <v>Invisible (Black hole)</v>
+        <v>Stellar Black hole</v>
       </c>
       <c r="AC7" s="110">
         <f t="shared" si="12"/>
@@ -4657,9 +4672,9 @@
         <f t="shared" si="10"/>
         <v>Invisible (Black hole)</v>
       </c>
-      <c r="AB8" s="104" t="str">
+      <c r="AB8" s="116" t="str">
         <f t="shared" si="11"/>
-        <v>Invisible (Black hole)</v>
+        <v>Invisible (geometric)</v>
       </c>
       <c r="AC8" s="110">
         <f t="shared" si="12"/>
@@ -4771,7 +4786,7 @@
         <f t="shared" si="10"/>
         <v>Partial visible</v>
       </c>
-      <c r="AB9" s="44" t="str">
+      <c r="AB9" s="117" t="str">
         <f t="shared" si="11"/>
         <v>Partial visible</v>
       </c>

</xml_diff>